<commit_message>
Update notes: 12-Sep-26 18:13:40.95
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSQF\Semester III\Time Series\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FFB607-E55E-4977-B6A4-2EB975FC0C46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2999F17-ED94-4B55-A7D4-60C378E95821}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Moving Average" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="07-09" sheetId="5" r:id="rId5"/>
     <sheet name="09-09" sheetId="7" r:id="rId6"/>
     <sheet name="10-09" sheetId="8" r:id="rId7"/>
+    <sheet name="11-09" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="74">
   <si>
     <t>Year</t>
   </si>
@@ -247,6 +248,18 @@
   </si>
   <si>
     <t>Ft</t>
+  </si>
+  <si>
+    <t>QUARTER</t>
+  </si>
+  <si>
+    <t>DSI</t>
+  </si>
+  <si>
+    <t>Qn AVG</t>
+  </si>
+  <si>
+    <t>RATIO-TO-MOVING-AVERAGE METHOD</t>
   </si>
 </sst>
 </file>
@@ -378,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -462,6 +475,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4985,4 +5001,402 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45A87D48-4F91-42E2-9B82-1240E1E85416}">
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" ht="15">
+      <c r="A1" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="29">
+        <v>4.8</v>
+      </c>
+      <c r="C3" s="29">
+        <f>J3/B16</f>
+        <v>0.90340136054421794</v>
+      </c>
+      <c r="D3" s="29">
+        <f>B3/C3</f>
+        <v>5.3132530120481913</v>
+      </c>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="31" t="s">
+        <v>72</v>
+      </c>
+      <c r="I3" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="33">
+        <f>(B3+B7+B11)/3</f>
+        <v>5.5333333333333341</v>
+      </c>
+      <c r="K3" s="29"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="29">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C4" s="29">
+        <f>J4/B16</f>
+        <v>0.8108843537414967</v>
+      </c>
+      <c r="D4" s="29">
+        <f t="shared" ref="D4:D14" si="0">B4/C4</f>
+        <v>5.0562080536912744</v>
+      </c>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="33">
+        <f>(B4+B8+B12)/3</f>
+        <v>4.9666666666666668</v>
+      </c>
+      <c r="K4" s="29"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="29">
+        <v>6</v>
+      </c>
+      <c r="C5" s="29">
+        <f>J5/B16</f>
+        <v>1.1047619047619048</v>
+      </c>
+      <c r="D5" s="29">
+        <f t="shared" si="0"/>
+        <v>5.4310344827586201</v>
+      </c>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="33">
+        <f>(B5+B9+B13)/3</f>
+        <v>6.7666666666666666</v>
+      </c>
+      <c r="K5" s="29"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="29">
+        <v>6.5</v>
+      </c>
+      <c r="C6" s="29">
+        <f>J6/B16</f>
+        <v>1.1809523809523812</v>
+      </c>
+      <c r="D6" s="29">
+        <f t="shared" si="0"/>
+        <v>5.5040322580645151</v>
+      </c>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="33">
+        <f>(B6+B10+B14)/3</f>
+        <v>7.2333333333333334</v>
+      </c>
+      <c r="K6" s="29"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="29">
+        <v>5.8</v>
+      </c>
+      <c r="C7" s="29">
+        <f>J3/B16</f>
+        <v>0.90340136054421794</v>
+      </c>
+      <c r="D7" s="29">
+        <f t="shared" si="0"/>
+        <v>6.4201807228915646</v>
+      </c>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+      <c r="J7" s="29"/>
+      <c r="K7" s="29"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="29">
+        <v>5.2</v>
+      </c>
+      <c r="C8" s="29">
+        <f>J4/B16</f>
+        <v>0.8108843537414967</v>
+      </c>
+      <c r="D8" s="29">
+        <f t="shared" si="0"/>
+        <v>6.4127516778523486</v>
+      </c>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="29"/>
+      <c r="K8" s="29"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="29">
+        <v>6.8</v>
+      </c>
+      <c r="C9" s="29">
+        <f>J5/B16</f>
+        <v>1.1047619047619048</v>
+      </c>
+      <c r="D9" s="29">
+        <f t="shared" si="0"/>
+        <v>6.1551724137931032</v>
+      </c>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" s="29">
+        <f>J3/B16</f>
+        <v>0.90340136054421794</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="29">
+        <v>7.4</v>
+      </c>
+      <c r="C10" s="29">
+        <f>J6/B16</f>
+        <v>1.1809523809523812</v>
+      </c>
+      <c r="D10" s="29">
+        <f t="shared" si="0"/>
+        <v>6.2661290322580632</v>
+      </c>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="29">
+        <f>J4/B16</f>
+        <v>0.8108843537414967</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="29">
+        <v>6</v>
+      </c>
+      <c r="C11" s="29">
+        <f>J3/B16</f>
+        <v>0.90340136054421794</v>
+      </c>
+      <c r="D11" s="29">
+        <f t="shared" si="0"/>
+        <v>6.6415662650602387</v>
+      </c>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="K11" s="29">
+        <f>J5/B16</f>
+        <v>1.1047619047619048</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="29">
+        <v>5.6</v>
+      </c>
+      <c r="C12" s="29">
+        <f>J4/B16</f>
+        <v>0.8108843537414967</v>
+      </c>
+      <c r="D12" s="29">
+        <f t="shared" si="0"/>
+        <v>6.9060402684563744</v>
+      </c>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="K12" s="29">
+        <f>J6/B16</f>
+        <v>1.1809523809523812</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="29">
+        <v>7.5</v>
+      </c>
+      <c r="C13" s="29">
+        <f>J5/B16</f>
+        <v>1.1047619047619048</v>
+      </c>
+      <c r="D13" s="29">
+        <f t="shared" si="0"/>
+        <v>6.7887931034482758</v>
+      </c>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+      <c r="J13" s="29"/>
+      <c r="K13" s="29"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="29">
+        <v>7.8</v>
+      </c>
+      <c r="C14" s="29">
+        <f>J6/B16</f>
+        <v>1.1809523809523812</v>
+      </c>
+      <c r="D14" s="29">
+        <f t="shared" si="0"/>
+        <v>6.6048387096774182</v>
+      </c>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
+      <c r="K14" s="29"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="29"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="29"/>
+      <c r="K15" s="29"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="29"/>
+      <c r="B16" s="29">
+        <f>AVERAGE(B3:B14)</f>
+        <v>6.1249999999999991</v>
+      </c>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+      <c r="J16" s="29"/>
+      <c r="K16" s="29"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="H3:H6"/>
+    <mergeCell ref="I9:I12"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update notes: 15-09-2026 19:47
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -471,13 +471,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4501,17 +4501,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
     </row>
     <row r="2" spans="1:9">
       <c r="B2" t="s">
@@ -4543,7 +4543,7 @@
       <c r="E3" s="28">
         <v>3.5</v>
       </c>
-      <c r="G3" s="31" t="s">
+      <c r="G3" s="32" t="s">
         <v>43</v>
       </c>
       <c r="H3" t="s">
@@ -4570,7 +4570,7 @@
       <c r="E4" s="28">
         <v>3.6</v>
       </c>
-      <c r="G4" s="31"/>
+      <c r="G4" s="32"/>
       <c r="H4" t="s">
         <v>24</v>
       </c>
@@ -4595,7 +4595,7 @@
       <c r="E5" s="28">
         <v>3.1</v>
       </c>
-      <c r="G5" s="31"/>
+      <c r="G5" s="32"/>
       <c r="H5" t="s">
         <v>26</v>
       </c>
@@ -4620,7 +4620,7 @@
       <c r="E6" s="28">
         <v>4</v>
       </c>
-      <c r="G6" s="31"/>
+      <c r="G6" s="32"/>
       <c r="H6" t="s">
         <v>28</v>
       </c>
@@ -4667,17 +4667,17 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="15">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
     </row>
     <row r="14" spans="1:9">
       <c r="B14" t="s">
@@ -4778,17 +4778,17 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="15">
-      <c r="A21" s="32" t="s">
+      <c r="A21" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="32"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="33"/>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="29" t="s">
@@ -4873,17 +4873,17 @@
       </c>
     </row>
     <row r="28" spans="1:9" ht="15">
-      <c r="A28" s="32" t="s">
+      <c r="A28" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="32"/>
+      <c r="B28" s="33"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="29" t="s">
@@ -5009,19 +5009,19 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="15">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="29" t="s">
@@ -5060,13 +5060,13 @@
       <c r="E3" s="29"/>
       <c r="F3" s="29"/>
       <c r="G3" s="29"/>
-      <c r="H3" s="31" t="s">
+      <c r="H3" s="32" t="s">
         <v>72</v>
       </c>
       <c r="I3" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="33">
+      <c r="J3" s="31">
         <f>(B3+B7+B11)/3</f>
         <v>5.5333333333333341</v>
       </c>
@@ -5090,11 +5090,11 @@
       <c r="E4" s="29"/>
       <c r="F4" s="29"/>
       <c r="G4" s="29"/>
-      <c r="H4" s="31"/>
+      <c r="H4" s="32"/>
       <c r="I4" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="33">
+      <c r="J4" s="31">
         <f>(B4+B8+B12)/3</f>
         <v>4.9666666666666668</v>
       </c>
@@ -5118,11 +5118,11 @@
       <c r="E5" s="29"/>
       <c r="F5" s="29"/>
       <c r="G5" s="29"/>
-      <c r="H5" s="31"/>
+      <c r="H5" s="32"/>
       <c r="I5" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="J5" s="33">
+      <c r="J5" s="31">
         <f>(B5+B9+B13)/3</f>
         <v>6.7666666666666666</v>
       </c>
@@ -5146,11 +5146,11 @@
       <c r="E6" s="29"/>
       <c r="F6" s="29"/>
       <c r="G6" s="29"/>
-      <c r="H6" s="31"/>
+      <c r="H6" s="32"/>
       <c r="I6" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="33">
+      <c r="J6" s="31">
         <f>(B6+B10+B14)/3</f>
         <v>7.2333333333333334</v>
       </c>
@@ -5221,7 +5221,7 @@
       <c r="F9" s="29"/>
       <c r="G9" s="29"/>
       <c r="H9" s="29"/>
-      <c r="I9" s="31" t="s">
+      <c r="I9" s="32" t="s">
         <v>43</v>
       </c>
       <c r="J9" s="29" t="s">
@@ -5251,7 +5251,7 @@
       <c r="F10" s="29"/>
       <c r="G10" s="29"/>
       <c r="H10" s="29"/>
-      <c r="I10" s="31"/>
+      <c r="I10" s="32"/>
       <c r="J10" s="29" t="s">
         <v>24</v>
       </c>
@@ -5279,7 +5279,7 @@
       <c r="F11" s="29"/>
       <c r="G11" s="29"/>
       <c r="H11" s="29"/>
-      <c r="I11" s="31"/>
+      <c r="I11" s="32"/>
       <c r="J11" s="29" t="s">
         <v>26</v>
       </c>
@@ -5307,7 +5307,7 @@
       <c r="F12" s="29"/>
       <c r="G12" s="29"/>
       <c r="H12" s="29"/>
-      <c r="I12" s="31"/>
+      <c r="I12" s="32"/>
       <c r="J12" s="29" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
feat(financial-math): add 17/09/2026 lecture on MM dividend irrelevance theory, Stewart Ltd problem, and Box 12 in formula reference
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSQF\Semester III\Time Series\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2999F17-ED94-4B55-A7D4-60C378E95821}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E3FA7A-9283-413A-8F47-5F78E7E945FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Moving Average" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="09-09" sheetId="7" r:id="rId6"/>
     <sheet name="10-09" sheetId="8" r:id="rId7"/>
     <sheet name="11-09" sheetId="9" r:id="rId8"/>
+    <sheet name="17-09" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="77">
   <si>
     <t>Year</t>
   </si>
@@ -260,6 +261,15 @@
   </si>
   <si>
     <t>RATIO-TO-MOVING-AVERAGE METHOD</t>
+  </si>
+  <si>
+    <t>Y1</t>
+  </si>
+  <si>
+    <t>Y2</t>
+  </si>
+  <si>
+    <t>Additive model</t>
   </si>
 </sst>
 </file>
@@ -1786,6 +1796,55 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>676956</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>171600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C20EE525-EDBE-D0C7-E9B4-22518ABF222A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6086475" y="0"/>
+          <a:ext cx="4877481" cy="1076475"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
@@ -5399,4 +5458,113 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5A482D-4E60-40E4-A3CA-59F54D2287F5}">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="26">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="32"/>
+      <c r="B3" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="26">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="32"/>
+      <c r="B4" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="26">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="32"/>
+      <c r="B5" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="26">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="26">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="32"/>
+      <c r="B7" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="26">
+        <v>130</v>
+      </c>
+      <c r="E7" s="26">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="32"/>
+      <c r="B8" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="26">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="32"/>
+      <c r="B9" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="26">
+        <v>140</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add GFM Section 1.9, Chapter 2 (Forex Market), Formula Reference Sheet, and Time Series notes (07/09 - 21/09/2026)
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSQF\Semester III\Time Series\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E3FA7A-9283-413A-8F47-5F78E7E945FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E253CE7-B103-4C84-B118-1BC5C4A989D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Moving Average" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="10-09" sheetId="8" r:id="rId7"/>
     <sheet name="11-09" sheetId="9" r:id="rId8"/>
     <sheet name="17-09" sheetId="10" r:id="rId9"/>
+    <sheet name="21-09" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="89">
   <si>
     <t>Year</t>
   </si>
@@ -270,6 +271,42 @@
   </si>
   <si>
     <t>Additive model</t>
+  </si>
+  <si>
+    <t>HW</t>
+  </si>
+  <si>
+    <t>H Method</t>
+  </si>
+  <si>
+    <t>sales</t>
+  </si>
+  <si>
+    <t>St</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>overall avg</t>
+  </si>
+  <si>
+    <t>SIQ1</t>
+  </si>
+  <si>
+    <t>SIQ2</t>
+  </si>
+  <si>
+    <t>SIQ3</t>
+  </si>
+  <si>
+    <t>SIQ4</t>
+  </si>
+  <si>
+    <t>TOTAL SI</t>
+  </si>
+  <si>
+    <t>DESEASONALISED DATA</t>
   </si>
 </sst>
 </file>
@@ -401,7 +438,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -489,6 +526,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2293,6 +2333,377 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{611D6F19-5A30-4094-86E7-5F0093F9B624}">
+  <dimension ref="A1:K18"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="12.375" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="11.375" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="9" style="8"/>
+    <col min="8" max="9" width="10.375" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.375" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.375" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="15">
+      <c r="A1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="6">
+        <v>2024</v>
+      </c>
+      <c r="B2" s="8">
+        <v>100</v>
+      </c>
+      <c r="C2" s="8">
+        <v>120</v>
+      </c>
+      <c r="D2" s="8">
+        <v>110</v>
+      </c>
+      <c r="E2" s="8">
+        <v>130</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="6">
+        <v>2025</v>
+      </c>
+      <c r="B3" s="8">
+        <v>110</v>
+      </c>
+      <c r="C3" s="8">
+        <v>130</v>
+      </c>
+      <c r="D3" s="8">
+        <v>120</v>
+      </c>
+      <c r="E3" s="8">
+        <v>140</v>
+      </c>
+      <c r="H3" s="8">
+        <v>80</v>
+      </c>
+      <c r="I3" s="8">
+        <f>H3</f>
+        <v>80</v>
+      </c>
+      <c r="J3" s="8">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="K3" s="8">
+        <f>H3</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="8">
+        <f>AVERAGE(B2:B3)</f>
+        <v>105</v>
+      </c>
+      <c r="C4" s="8">
+        <f t="shared" ref="C4:E4" si="0">AVERAGE(C2:C3)</f>
+        <v>125</v>
+      </c>
+      <c r="D4" s="8">
+        <f t="shared" si="0"/>
+        <v>115</v>
+      </c>
+      <c r="E4" s="8">
+        <f t="shared" si="0"/>
+        <v>135</v>
+      </c>
+      <c r="H4" s="8">
+        <v>82</v>
+      </c>
+      <c r="I4" s="8">
+        <f>0.5*(H4)+(1-0.5)*(I3+J3)</f>
+        <v>81</v>
+      </c>
+      <c r="J4" s="8">
+        <f>0.5*(I4-I3)+(1-0.5)*J3</f>
+        <v>0.5</v>
+      </c>
+      <c r="K4" s="8">
+        <f>I4+J4</f>
+        <v>81.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="H5" s="8">
+        <v>84</v>
+      </c>
+      <c r="I5" s="8">
+        <f>0.5*(H5)+(1-0.5)*(I4+J4)</f>
+        <v>82.75</v>
+      </c>
+      <c r="J5" s="8">
+        <f>0.5*(I5-I4)+(1-0.5)*J4</f>
+        <v>1.125</v>
+      </c>
+      <c r="K5" s="8">
+        <f>I5+J5</f>
+        <v>83.875</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="8">
+        <f>AVERAGE(B2:E3)</f>
+        <v>120</v>
+      </c>
+      <c r="H6" s="8">
+        <v>89</v>
+      </c>
+      <c r="I6" s="8">
+        <f>0.5*(H6)+(1-0.5)*(I5+J5)</f>
+        <v>86.4375</v>
+      </c>
+      <c r="J6" s="8">
+        <f>0.5*(I6-I5)+(1-0.5)*J5</f>
+        <v>2.40625</v>
+      </c>
+      <c r="K6" s="8">
+        <f>I6+J6</f>
+        <v>88.84375</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="H7" s="8">
+        <v>90</v>
+      </c>
+      <c r="I7" s="8">
+        <f>0.5*(H7)+(1-0.5)*(I6+J6)</f>
+        <v>89.421875</v>
+      </c>
+      <c r="J7" s="8">
+        <f>0.5*(I7-I6)+(1-0.5)*J6</f>
+        <v>2.6953125</v>
+      </c>
+      <c r="K7" s="8">
+        <f>I7+J7</f>
+        <v>92.1171875</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="8">
+        <f>B4/$B$6</f>
+        <v>0.875</v>
+      </c>
+      <c r="H8" s="8">
+        <v>91</v>
+      </c>
+      <c r="I8" s="8">
+        <f>0.5*(H8)+(1-0.5)*(I7+J7)</f>
+        <v>91.55859375</v>
+      </c>
+      <c r="J8" s="8">
+        <f>0.5*(I8-I7)+(1-0.5)*J7</f>
+        <v>2.416015625</v>
+      </c>
+      <c r="K8" s="8">
+        <f>I8+J8</f>
+        <v>93.974609375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="8">
+        <f>C4/B6</f>
+        <v>1.0416666666666667</v>
+      </c>
+      <c r="H9" s="8">
+        <v>95</v>
+      </c>
+      <c r="I9" s="8">
+        <f>0.5*(H9)+(1-0.5)*(I8+J8)</f>
+        <v>94.4873046875</v>
+      </c>
+      <c r="J9" s="8">
+        <f>0.5*(I9-I8)+(1-0.5)*J8</f>
+        <v>2.67236328125</v>
+      </c>
+      <c r="K9" s="8">
+        <f>I9+J9</f>
+        <v>97.15966796875</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="8">
+        <f>D4/B6</f>
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="H10" s="8">
+        <v>98</v>
+      </c>
+      <c r="I10" s="8">
+        <f>0.5*(H10)+(1-0.5)*(I9+J9)</f>
+        <v>97.579833984375</v>
+      </c>
+      <c r="J10" s="8">
+        <f>0.5*(I10-I9)+(1-0.5)*J9</f>
+        <v>2.8824462890625</v>
+      </c>
+      <c r="K10" s="8">
+        <f>I10+J10</f>
+        <v>100.4622802734375</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="8">
+        <f>E4/B6</f>
+        <v>1.125</v>
+      </c>
+      <c r="H11" s="8">
+        <v>99</v>
+      </c>
+      <c r="I11" s="8">
+        <f>0.5*(H11)+(1-0.5)*(I10+J10)</f>
+        <v>99.73114013671875</v>
+      </c>
+      <c r="J11" s="8">
+        <f>0.5*(I11-I10)+(1-0.5)*J10</f>
+        <v>2.516876220703125</v>
+      </c>
+      <c r="K11" s="8">
+        <f>I11+J11</f>
+        <v>102.24801635742188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="8">
+        <f>SUM(B8:B12)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15">
+      <c r="A15" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="B16" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="6">
+        <v>2024</v>
+      </c>
+      <c r="B17" s="8">
+        <f>B2/B8</f>
+        <v>114.28571428571429</v>
+      </c>
+      <c r="C17" s="8">
+        <f>C2/B9</f>
+        <v>115.19999999999999</v>
+      </c>
+      <c r="D17" s="8">
+        <f>D2/B10</f>
+        <v>114.78260869565217</v>
+      </c>
+      <c r="E17" s="8">
+        <f>E2/B11</f>
+        <v>115.55555555555556</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="6">
+        <v>2025</v>
+      </c>
+      <c r="B18" s="8">
+        <f>B3/B8</f>
+        <v>125.71428571428571</v>
+      </c>
+      <c r="C18" s="8">
+        <f>C3/B9</f>
+        <v>124.8</v>
+      </c>
+      <c r="D18" s="8">
+        <f>D3/B10</f>
+        <v>125.21739130434783</v>
+      </c>
+      <c r="E18" s="8">
+        <f>E3/B11</f>
+        <v>124.44444444444444</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="H1:K1"/>
+    <mergeCell ref="A15:E15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9EF010B-22A5-42D6-BCC8-2D4478E9E621}">
   <dimension ref="C1:Y26"/>

</xml_diff>

<commit_message>
Update notes: 24-09-2026 19:46
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSQF\Semester III\Time Series\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E253CE7-B103-4C84-B118-1BC5C4A989D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6150FC8A-F57D-476E-9856-1AF55EB1A332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Moving Average" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="11-09" sheetId="9" r:id="rId8"/>
     <sheet name="17-09" sheetId="10" r:id="rId9"/>
     <sheet name="21-09" sheetId="11" r:id="rId10"/>
+    <sheet name="22-09" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="105">
   <si>
     <t>Year</t>
   </si>
@@ -307,17 +308,66 @@
   </si>
   <si>
     <t>DESEASONALISED DATA</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>xy</t>
+  </si>
+  <si>
+    <t>x^2</t>
+  </si>
+  <si>
+    <t>ycapt</t>
+  </si>
+  <si>
+    <t>(yt-ytcap)^2</t>
+  </si>
+  <si>
+    <t>(yt-ytbar)^2</t>
+  </si>
+  <si>
+    <t>MAPE</t>
+  </si>
+  <si>
+    <t>MAD</t>
+  </si>
+  <si>
+    <t>MSD</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>Yt bar</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R^2 = </t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>for year 2026 (x = 6)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -340,6 +390,30 @@
     <font>
       <sz val="10"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -438,7 +512,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -521,14 +595,51 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2363,12 +2474,12 @@
       <c r="E1" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="32" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="6">
@@ -2455,15 +2566,15 @@
         <v>82</v>
       </c>
       <c r="I4" s="8">
-        <f>0.5*(H4)+(1-0.5)*(I3+J3)</f>
+        <f t="shared" ref="I4:I11" si="1">0.5*(H4)+(1-0.5)*(I3+J3)</f>
         <v>81</v>
       </c>
       <c r="J4" s="8">
-        <f>0.5*(I4-I3)+(1-0.5)*J3</f>
+        <f t="shared" ref="J4:J11" si="2">0.5*(I4-I3)+(1-0.5)*J3</f>
         <v>0.5</v>
       </c>
       <c r="K4" s="8">
-        <f>I4+J4</f>
+        <f t="shared" ref="K4:K11" si="3">I4+J4</f>
         <v>81.5</v>
       </c>
     </row>
@@ -2472,15 +2583,15 @@
         <v>84</v>
       </c>
       <c r="I5" s="8">
-        <f>0.5*(H5)+(1-0.5)*(I4+J4)</f>
+        <f t="shared" si="1"/>
         <v>82.75</v>
       </c>
       <c r="J5" s="8">
-        <f>0.5*(I5-I4)+(1-0.5)*J4</f>
+        <f t="shared" si="2"/>
         <v>1.125</v>
       </c>
       <c r="K5" s="8">
-        <f>I5+J5</f>
+        <f t="shared" si="3"/>
         <v>83.875</v>
       </c>
     </row>
@@ -2496,15 +2607,15 @@
         <v>89</v>
       </c>
       <c r="I6" s="8">
-        <f>0.5*(H6)+(1-0.5)*(I5+J5)</f>
+        <f t="shared" si="1"/>
         <v>86.4375</v>
       </c>
       <c r="J6" s="8">
-        <f>0.5*(I6-I5)+(1-0.5)*J5</f>
+        <f t="shared" si="2"/>
         <v>2.40625</v>
       </c>
       <c r="K6" s="8">
-        <f>I6+J6</f>
+        <f t="shared" si="3"/>
         <v>88.84375</v>
       </c>
     </row>
@@ -2513,15 +2624,15 @@
         <v>90</v>
       </c>
       <c r="I7" s="8">
-        <f>0.5*(H7)+(1-0.5)*(I6+J6)</f>
+        <f t="shared" si="1"/>
         <v>89.421875</v>
       </c>
       <c r="J7" s="8">
-        <f>0.5*(I7-I6)+(1-0.5)*J6</f>
+        <f t="shared" si="2"/>
         <v>2.6953125</v>
       </c>
       <c r="K7" s="8">
-        <f>I7+J7</f>
+        <f t="shared" si="3"/>
         <v>92.1171875</v>
       </c>
     </row>
@@ -2537,15 +2648,15 @@
         <v>91</v>
       </c>
       <c r="I8" s="8">
-        <f>0.5*(H8)+(1-0.5)*(I7+J7)</f>
+        <f t="shared" si="1"/>
         <v>91.55859375</v>
       </c>
       <c r="J8" s="8">
-        <f>0.5*(I8-I7)+(1-0.5)*J7</f>
+        <f t="shared" si="2"/>
         <v>2.416015625</v>
       </c>
       <c r="K8" s="8">
-        <f>I8+J8</f>
+        <f t="shared" si="3"/>
         <v>93.974609375</v>
       </c>
     </row>
@@ -2561,15 +2672,15 @@
         <v>95</v>
       </c>
       <c r="I9" s="8">
-        <f>0.5*(H9)+(1-0.5)*(I8+J8)</f>
+        <f t="shared" si="1"/>
         <v>94.4873046875</v>
       </c>
       <c r="J9" s="8">
-        <f>0.5*(I9-I8)+(1-0.5)*J8</f>
+        <f t="shared" si="2"/>
         <v>2.67236328125</v>
       </c>
       <c r="K9" s="8">
-        <f>I9+J9</f>
+        <f t="shared" si="3"/>
         <v>97.15966796875</v>
       </c>
     </row>
@@ -2585,15 +2696,15 @@
         <v>98</v>
       </c>
       <c r="I10" s="8">
-        <f>0.5*(H10)+(1-0.5)*(I9+J9)</f>
+        <f t="shared" si="1"/>
         <v>97.579833984375</v>
       </c>
       <c r="J10" s="8">
-        <f>0.5*(I10-I9)+(1-0.5)*J9</f>
+        <f t="shared" si="2"/>
         <v>2.8824462890625</v>
       </c>
       <c r="K10" s="8">
-        <f>I10+J10</f>
+        <f t="shared" si="3"/>
         <v>100.4622802734375</v>
       </c>
     </row>
@@ -2609,15 +2720,15 @@
         <v>99</v>
       </c>
       <c r="I11" s="8">
-        <f>0.5*(H11)+(1-0.5)*(I10+J10)</f>
+        <f t="shared" si="1"/>
         <v>99.73114013671875</v>
       </c>
       <c r="J11" s="8">
-        <f>0.5*(I11-I10)+(1-0.5)*J10</f>
+        <f t="shared" si="2"/>
         <v>2.516876220703125</v>
       </c>
       <c r="K11" s="8">
-        <f>I11+J11</f>
+        <f t="shared" si="3"/>
         <v>102.24801635742188</v>
       </c>
     </row>
@@ -2631,13 +2742,13 @@
       </c>
     </row>
     <row r="15" spans="1:11" ht="15">
-      <c r="A15" s="34" t="s">
+      <c r="A15" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
     </row>
     <row r="16" spans="1:11">
       <c r="B16" s="8" t="s">
@@ -2700,6 +2811,457 @@
     <mergeCell ref="H1:K1"/>
     <mergeCell ref="A15:E15"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61FD1641-1B4A-46DC-8E88-B3C77646F907}">
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.25" style="42" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.875" style="42" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="6.875" style="42" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.875" style="42" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" style="42" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13" style="42" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.875" style="42" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="3.875" style="42" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.875" style="42" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="42"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="F1" s="35" t="s">
+        <v>93</v>
+      </c>
+      <c r="G1" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="H1" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="I1" s="35" t="s">
+        <v>96</v>
+      </c>
+      <c r="J1" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="K1" s="35" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="35">
+        <v>2021</v>
+      </c>
+      <c r="B2" s="35">
+        <v>1</v>
+      </c>
+      <c r="C2" s="35">
+        <v>22600</v>
+      </c>
+      <c r="D2" s="35">
+        <f>B2*C2</f>
+        <v>22600</v>
+      </c>
+      <c r="E2" s="35">
+        <f>B2^2</f>
+        <v>1</v>
+      </c>
+      <c r="F2" s="43">
+        <f>-235*B2+22860</f>
+        <v>22625</v>
+      </c>
+      <c r="G2" s="43">
+        <f>(C2-F2)^2</f>
+        <v>625</v>
+      </c>
+      <c r="H2" s="43">
+        <f>(C2-$B$9)^2</f>
+        <v>198025</v>
+      </c>
+      <c r="I2" s="44">
+        <f>(100/$B$8)*ABS(C2-F2)/C2</f>
+        <v>2.2123893805309734E-2</v>
+      </c>
+      <c r="J2" s="43">
+        <f>(1/$B$8)*ABS(C2-F2)</f>
+        <v>5</v>
+      </c>
+      <c r="K2" s="43">
+        <f>(1/$B$8)*ABS(C2-F2)^2</f>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="35">
+        <v>2022</v>
+      </c>
+      <c r="B3" s="35">
+        <v>2</v>
+      </c>
+      <c r="C3" s="35">
+        <v>22400</v>
+      </c>
+      <c r="D3" s="35">
+        <f t="shared" ref="D3:D6" si="0">B3*C3</f>
+        <v>44800</v>
+      </c>
+      <c r="E3" s="35">
+        <f t="shared" ref="E3:E6" si="1">B3^2</f>
+        <v>4</v>
+      </c>
+      <c r="F3" s="43">
+        <f>-235*B3+22860</f>
+        <v>22390</v>
+      </c>
+      <c r="G3" s="43">
+        <f t="shared" ref="G3:G6" si="2">(C3-F3)^2</f>
+        <v>100</v>
+      </c>
+      <c r="H3" s="43">
+        <f t="shared" ref="H3:H11" si="3">(C3-$B$9)^2</f>
+        <v>60025</v>
+      </c>
+      <c r="I3" s="44">
+        <f>(100/$B$8)*ABS(C3-F3)/C3</f>
+        <v>8.9285714285714281E-3</v>
+      </c>
+      <c r="J3" s="43">
+        <f>(1/$B$8)*ABS(C3-F3)</f>
+        <v>2</v>
+      </c>
+      <c r="K3" s="43">
+        <f>(1/$B$8)*ABS(C3-F3)^2</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="35">
+        <v>2023</v>
+      </c>
+      <c r="B4" s="35">
+        <v>3</v>
+      </c>
+      <c r="C4" s="35">
+        <v>22250</v>
+      </c>
+      <c r="D4" s="35">
+        <f t="shared" si="0"/>
+        <v>66750</v>
+      </c>
+      <c r="E4" s="35">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="F4" s="43">
+        <f>-235*B4+22860</f>
+        <v>22155</v>
+      </c>
+      <c r="G4" s="43">
+        <f t="shared" si="2"/>
+        <v>9025</v>
+      </c>
+      <c r="H4" s="43">
+        <f t="shared" si="3"/>
+        <v>9025</v>
+      </c>
+      <c r="I4" s="44">
+        <f>(100/$B$8)*ABS(C4-F4)/C4</f>
+        <v>8.5393258426966295E-2</v>
+      </c>
+      <c r="J4" s="43">
+        <f>(1/$B$8)*ABS(C4-F4)</f>
+        <v>19</v>
+      </c>
+      <c r="K4" s="43">
+        <f>(1/$B$8)*ABS(C4-F4)^2</f>
+        <v>1805</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="35">
+        <v>2024</v>
+      </c>
+      <c r="B5" s="35">
+        <v>4</v>
+      </c>
+      <c r="C5" s="35">
+        <v>21800</v>
+      </c>
+      <c r="D5" s="35">
+        <f t="shared" si="0"/>
+        <v>87200</v>
+      </c>
+      <c r="E5" s="35">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="F5" s="43">
+        <f>-235*B5+22860</f>
+        <v>21920</v>
+      </c>
+      <c r="G5" s="43">
+        <f t="shared" si="2"/>
+        <v>14400</v>
+      </c>
+      <c r="H5" s="43">
+        <f t="shared" si="3"/>
+        <v>126025</v>
+      </c>
+      <c r="I5" s="44">
+        <f>(100/$B$8)*ABS(C5-F5)/C5</f>
+        <v>0.11009174311926606</v>
+      </c>
+      <c r="J5" s="43">
+        <f>(1/$B$8)*ABS(C5-F5)</f>
+        <v>24</v>
+      </c>
+      <c r="K5" s="43">
+        <f>(1/$B$8)*ABS(C5-F5)^2</f>
+        <v>2880</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="35">
+        <v>2025</v>
+      </c>
+      <c r="B6" s="35">
+        <v>5</v>
+      </c>
+      <c r="C6" s="35">
+        <v>21725</v>
+      </c>
+      <c r="D6" s="35">
+        <f t="shared" si="0"/>
+        <v>108625</v>
+      </c>
+      <c r="E6" s="35">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="F6" s="43">
+        <f>-235*B6+22860</f>
+        <v>21685</v>
+      </c>
+      <c r="G6" s="43">
+        <f t="shared" si="2"/>
+        <v>1600</v>
+      </c>
+      <c r="H6" s="43">
+        <f t="shared" si="3"/>
+        <v>184900</v>
+      </c>
+      <c r="I6" s="44">
+        <f>(100/$B$8)*ABS(C6-F6)/C6</f>
+        <v>3.6823935558112773E-2</v>
+      </c>
+      <c r="J6" s="43">
+        <f>(1/$B$8)*ABS(C6-F6)</f>
+        <v>8</v>
+      </c>
+      <c r="K6" s="43">
+        <f>(1/$B$8)*ABS(C6-F6)^2</f>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="36">
+        <f>SUM(B2:B6)</f>
+        <v>15</v>
+      </c>
+      <c r="C7" s="36">
+        <f>SUM(C2:C6)</f>
+        <v>110775</v>
+      </c>
+      <c r="D7" s="36">
+        <f>SUM(D2:D6)</f>
+        <v>329975</v>
+      </c>
+      <c r="E7" s="36">
+        <f>SUM(E2:E6)</f>
+        <v>55</v>
+      </c>
+      <c r="F7" s="45"/>
+      <c r="G7" s="45">
+        <f>SUM(G2:G6)</f>
+        <v>25750</v>
+      </c>
+      <c r="H7" s="45">
+        <f>SUM(H2:H6)</f>
+        <v>578000</v>
+      </c>
+      <c r="I7" s="37">
+        <f>SUM(I2:I6)</f>
+        <v>0.2633614023382263</v>
+      </c>
+      <c r="J7" s="45">
+        <f>SUM(J2:J6)</f>
+        <v>58</v>
+      </c>
+      <c r="K7" s="45">
+        <f>SUM(K2:K6)</f>
+        <v>5150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="B8" s="38">
+        <f>COUNT(B2:B6)</f>
+        <v>5</v>
+      </c>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="46"/>
+      <c r="J8" s="46"/>
+      <c r="K8" s="46"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" s="38">
+        <f>AVERAGE(C2:C6)</f>
+        <v>22155</v>
+      </c>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
+      <c r="J9" s="46"/>
+      <c r="K9" s="46"/>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="B10" s="39">
+        <f>(B8*D7-B7*C7)/(B8*E7-B7^2)</f>
+        <v>-235</v>
+      </c>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="G10" s="46">
+        <f>1-(G7/H7)</f>
+        <v>0.95544982698961933</v>
+      </c>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="46"/>
+      <c r="K10" s="46"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" s="39">
+        <f>(C7-B10*B7)/(B8)</f>
+        <v>22860</v>
+      </c>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
+      <c r="I11" s="46"/>
+      <c r="J11" s="46"/>
+      <c r="K11" s="46"/>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="40"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="47"/>
+      <c r="J12" s="47"/>
+      <c r="K12" s="47"/>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="41" t="s">
+        <v>104</v>
+      </c>
+      <c r="B13" s="40"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="47"/>
+      <c r="G13" s="47"/>
+      <c r="H13" s="47"/>
+      <c r="I13" s="47"/>
+      <c r="J13" s="47"/>
+      <c r="K13" s="47"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="41" t="str">
+        <f>"y = "&amp;B11&amp;"+"&amp;B10&amp;"x"</f>
+        <v>y = 22860+-235x</v>
+      </c>
+      <c r="B14" s="40"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="41" t="str">
+        <f>"y = "&amp;B11+B10*(6)</f>
+        <v>y = 21450</v>
+      </c>
+      <c r="B15" s="40"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="47"/>
+      <c r="K15" s="47"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4971,17 +5533,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
     </row>
     <row r="2" spans="1:9">
       <c r="B2" t="s">
@@ -5013,7 +5575,7 @@
       <c r="E3" s="28">
         <v>3.5</v>
       </c>
-      <c r="G3" s="32" t="s">
+      <c r="G3" s="33" t="s">
         <v>43</v>
       </c>
       <c r="H3" t="s">
@@ -5040,7 +5602,7 @@
       <c r="E4" s="28">
         <v>3.6</v>
       </c>
-      <c r="G4" s="32"/>
+      <c r="G4" s="33"/>
       <c r="H4" t="s">
         <v>24</v>
       </c>
@@ -5065,7 +5627,7 @@
       <c r="E5" s="28">
         <v>3.1</v>
       </c>
-      <c r="G5" s="32"/>
+      <c r="G5" s="33"/>
       <c r="H5" t="s">
         <v>26</v>
       </c>
@@ -5090,7 +5652,7 @@
       <c r="E6" s="28">
         <v>4</v>
       </c>
-      <c r="G6" s="32"/>
+      <c r="G6" s="33"/>
       <c r="H6" t="s">
         <v>28</v>
       </c>
@@ -5137,17 +5699,17 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="15">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="33"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="33"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="33"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="34"/>
     </row>
     <row r="14" spans="1:9">
       <c r="B14" t="s">
@@ -5248,17 +5810,17 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="15">
-      <c r="A21" s="33" t="s">
+      <c r="A21" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="B21" s="33"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="33"/>
-      <c r="I21" s="33"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="34"/>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="29" t="s">
@@ -5343,17 +5905,17 @@
       </c>
     </row>
     <row r="28" spans="1:9" ht="15">
-      <c r="A28" s="33" t="s">
+      <c r="A28" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
+      <c r="I28" s="34"/>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="29" t="s">
@@ -5479,19 +6041,19 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="15">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="29" t="s">
@@ -5530,7 +6092,7 @@
       <c r="E3" s="29"/>
       <c r="F3" s="29"/>
       <c r="G3" s="29"/>
-      <c r="H3" s="32" t="s">
+      <c r="H3" s="33" t="s">
         <v>72</v>
       </c>
       <c r="I3" s="29" t="s">
@@ -5560,7 +6122,7 @@
       <c r="E4" s="29"/>
       <c r="F4" s="29"/>
       <c r="G4" s="29"/>
-      <c r="H4" s="32"/>
+      <c r="H4" s="33"/>
       <c r="I4" s="29" t="s">
         <v>24</v>
       </c>
@@ -5588,7 +6150,7 @@
       <c r="E5" s="29"/>
       <c r="F5" s="29"/>
       <c r="G5" s="29"/>
-      <c r="H5" s="32"/>
+      <c r="H5" s="33"/>
       <c r="I5" s="29" t="s">
         <v>26</v>
       </c>
@@ -5616,7 +6178,7 @@
       <c r="E6" s="29"/>
       <c r="F6" s="29"/>
       <c r="G6" s="29"/>
-      <c r="H6" s="32"/>
+      <c r="H6" s="33"/>
       <c r="I6" s="29" t="s">
         <v>28</v>
       </c>
@@ -5691,7 +6253,7 @@
       <c r="F9" s="29"/>
       <c r="G9" s="29"/>
       <c r="H9" s="29"/>
-      <c r="I9" s="32" t="s">
+      <c r="I9" s="33" t="s">
         <v>43</v>
       </c>
       <c r="J9" s="29" t="s">
@@ -5721,7 +6283,7 @@
       <c r="F10" s="29"/>
       <c r="G10" s="29"/>
       <c r="H10" s="29"/>
-      <c r="I10" s="32"/>
+      <c r="I10" s="33"/>
       <c r="J10" s="29" t="s">
         <v>24</v>
       </c>
@@ -5749,7 +6311,7 @@
       <c r="F11" s="29"/>
       <c r="G11" s="29"/>
       <c r="H11" s="29"/>
-      <c r="I11" s="32"/>
+      <c r="I11" s="33"/>
       <c r="J11" s="29" t="s">
         <v>26</v>
       </c>
@@ -5777,7 +6339,7 @@
       <c r="F12" s="29"/>
       <c r="G12" s="29"/>
       <c r="H12" s="29"/>
-      <c r="I12" s="32"/>
+      <c r="I12" s="33"/>
       <c r="J12" s="29" t="s">
         <v>28</v>
       </c>
@@ -5880,17 +6442,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>74</v>
       </c>
       <c r="B2" s="26" t="s">
@@ -5901,7 +6463,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="32"/>
+      <c r="A3" s="33"/>
       <c r="B3" s="26" t="s">
         <v>24</v>
       </c>
@@ -5910,7 +6472,7 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="32"/>
+      <c r="A4" s="33"/>
       <c r="B4" s="26" t="s">
         <v>26</v>
       </c>
@@ -5919,7 +6481,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="32"/>
+      <c r="A5" s="33"/>
       <c r="B5" s="26" t="s">
         <v>28</v>
       </c>
@@ -5928,7 +6490,7 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="33" t="s">
         <v>75</v>
       </c>
       <c r="B6" s="26" t="s">
@@ -5939,7 +6501,7 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="32"/>
+      <c r="A7" s="33"/>
       <c r="B7" s="26" t="s">
         <v>24</v>
       </c>
@@ -5951,7 +6513,7 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="32"/>
+      <c r="A8" s="33"/>
       <c r="B8" s="26" t="s">
         <v>26</v>
       </c>
@@ -5960,7 +6522,7 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="32"/>
+      <c r="A9" s="33"/>
       <c r="B9" s="26" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
feat(fin-math): initiate Chapter 3, update formula reference sheet (Boxes 13-17), and sync docs (Lectures 22/09-13/10/2026)
</commit_message>
<xml_diff>
--- a/Time Series/moving_average.xlsx
+++ b/Time Series/moving_average.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSQF\Semester III\Time Series\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6150FC8A-F57D-476E-9856-1AF55EB1A332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D0A49B-0B0F-4FD4-9184-3C94FFA229C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Moving Average" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="17-09" sheetId="10" r:id="rId9"/>
     <sheet name="21-09" sheetId="11" r:id="rId10"/>
     <sheet name="22-09" sheetId="12" r:id="rId11"/>
+    <sheet name="08-10" sheetId="13" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="107">
   <si>
     <t>Year</t>
   </si>
@@ -356,6 +357,12 @@
   </si>
   <si>
     <t>for year 2026 (x = 6)</t>
+  </si>
+  <si>
+    <t>yt</t>
+  </si>
+  <si>
+    <t>yt-yt-1</t>
   </si>
 </sst>
 </file>
@@ -595,15 +602,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -640,6 +638,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2474,12 +2481,12 @@
       <c r="E1" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="6">
@@ -2742,13 +2749,13 @@
       </c>
     </row>
     <row r="15" spans="1:11" ht="15">
-      <c r="A15" s="32" t="s">
+      <c r="A15" s="47" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47"/>
     </row>
     <row r="16" spans="1:11">
       <c r="B16" s="8" t="s">
@@ -2820,446 +2827,579 @@
   <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.25" style="42" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.875" style="42" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="6.875" style="42" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="3.875" style="42" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6" style="42" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="13" style="42" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.875" style="42" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="3.875" style="42" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.875" style="42" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9" style="42"/>
+    <col min="1" max="1" width="22.25" style="39" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.875" style="39" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="6.875" style="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.875" style="39" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" style="39" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13" style="39" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.875" style="39" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="3.875" style="39" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.875" style="39" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="32" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="F1" s="32" t="s">
         <v>93</v>
       </c>
-      <c r="G1" s="35" t="s">
+      <c r="G1" s="32" t="s">
         <v>94</v>
       </c>
-      <c r="H1" s="35" t="s">
+      <c r="H1" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="I1" s="35" t="s">
+      <c r="I1" s="32" t="s">
         <v>96</v>
       </c>
-      <c r="J1" s="35" t="s">
+      <c r="J1" s="32" t="s">
         <v>97</v>
       </c>
-      <c r="K1" s="35" t="s">
+      <c r="K1" s="32" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="35">
+      <c r="A2" s="32">
         <v>2021</v>
       </c>
-      <c r="B2" s="35">
+      <c r="B2" s="32">
         <v>1</v>
       </c>
-      <c r="C2" s="35">
+      <c r="C2" s="32">
         <v>22600</v>
       </c>
-      <c r="D2" s="35">
+      <c r="D2" s="32">
         <f>B2*C2</f>
         <v>22600</v>
       </c>
-      <c r="E2" s="35">
+      <c r="E2" s="32">
         <f>B2^2</f>
         <v>1</v>
       </c>
-      <c r="F2" s="43">
+      <c r="F2" s="40">
         <f>-235*B2+22860</f>
         <v>22625</v>
       </c>
-      <c r="G2" s="43">
+      <c r="G2" s="40">
         <f>(C2-F2)^2</f>
         <v>625</v>
       </c>
-      <c r="H2" s="43">
+      <c r="H2" s="40">
         <f>(C2-$B$9)^2</f>
         <v>198025</v>
       </c>
-      <c r="I2" s="44">
+      <c r="I2" s="41">
         <f>(100/$B$8)*ABS(C2-F2)/C2</f>
         <v>2.2123893805309734E-2</v>
       </c>
-      <c r="J2" s="43">
+      <c r="J2" s="40">
         <f>(1/$B$8)*ABS(C2-F2)</f>
         <v>5</v>
       </c>
-      <c r="K2" s="43">
+      <c r="K2" s="40">
         <f>(1/$B$8)*ABS(C2-F2)^2</f>
         <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="35">
+      <c r="A3" s="32">
         <v>2022</v>
       </c>
-      <c r="B3" s="35">
+      <c r="B3" s="32">
         <v>2</v>
       </c>
-      <c r="C3" s="35">
+      <c r="C3" s="32">
         <v>22400</v>
       </c>
-      <c r="D3" s="35">
+      <c r="D3" s="32">
         <f t="shared" ref="D3:D6" si="0">B3*C3</f>
         <v>44800</v>
       </c>
-      <c r="E3" s="35">
+      <c r="E3" s="32">
         <f t="shared" ref="E3:E6" si="1">B3^2</f>
         <v>4</v>
       </c>
-      <c r="F3" s="43">
+      <c r="F3" s="40">
         <f>-235*B3+22860</f>
         <v>22390</v>
       </c>
-      <c r="G3" s="43">
+      <c r="G3" s="40">
         <f t="shared" ref="G3:G6" si="2">(C3-F3)^2</f>
         <v>100</v>
       </c>
-      <c r="H3" s="43">
-        <f t="shared" ref="H3:H11" si="3">(C3-$B$9)^2</f>
+      <c r="H3" s="40">
+        <f t="shared" ref="H3:H6" si="3">(C3-$B$9)^2</f>
         <v>60025</v>
       </c>
-      <c r="I3" s="44">
+      <c r="I3" s="41">
         <f>(100/$B$8)*ABS(C3-F3)/C3</f>
         <v>8.9285714285714281E-3</v>
       </c>
-      <c r="J3" s="43">
+      <c r="J3" s="40">
         <f>(1/$B$8)*ABS(C3-F3)</f>
         <v>2</v>
       </c>
-      <c r="K3" s="43">
+      <c r="K3" s="40">
         <f>(1/$B$8)*ABS(C3-F3)^2</f>
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="35">
+      <c r="A4" s="32">
         <v>2023</v>
       </c>
-      <c r="B4" s="35">
+      <c r="B4" s="32">
         <v>3</v>
       </c>
-      <c r="C4" s="35">
+      <c r="C4" s="32">
         <v>22250</v>
       </c>
-      <c r="D4" s="35">
+      <c r="D4" s="32">
         <f t="shared" si="0"/>
         <v>66750</v>
       </c>
-      <c r="E4" s="35">
+      <c r="E4" s="32">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="F4" s="43">
+      <c r="F4" s="40">
         <f>-235*B4+22860</f>
         <v>22155</v>
       </c>
-      <c r="G4" s="43">
+      <c r="G4" s="40">
         <f t="shared" si="2"/>
         <v>9025</v>
       </c>
-      <c r="H4" s="43">
+      <c r="H4" s="40">
         <f t="shared" si="3"/>
         <v>9025</v>
       </c>
-      <c r="I4" s="44">
+      <c r="I4" s="41">
         <f>(100/$B$8)*ABS(C4-F4)/C4</f>
         <v>8.5393258426966295E-2</v>
       </c>
-      <c r="J4" s="43">
+      <c r="J4" s="40">
         <f>(1/$B$8)*ABS(C4-F4)</f>
         <v>19</v>
       </c>
-      <c r="K4" s="43">
+      <c r="K4" s="40">
         <f>(1/$B$8)*ABS(C4-F4)^2</f>
         <v>1805</v>
       </c>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="35">
+      <c r="A5" s="32">
         <v>2024</v>
       </c>
-      <c r="B5" s="35">
+      <c r="B5" s="32">
         <v>4</v>
       </c>
-      <c r="C5" s="35">
+      <c r="C5" s="32">
         <v>21800</v>
       </c>
-      <c r="D5" s="35">
+      <c r="D5" s="32">
         <f t="shared" si="0"/>
         <v>87200</v>
       </c>
-      <c r="E5" s="35">
+      <c r="E5" s="32">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="F5" s="43">
+      <c r="F5" s="40">
         <f>-235*B5+22860</f>
         <v>21920</v>
       </c>
-      <c r="G5" s="43">
+      <c r="G5" s="40">
         <f t="shared" si="2"/>
         <v>14400</v>
       </c>
-      <c r="H5" s="43">
+      <c r="H5" s="40">
         <f t="shared" si="3"/>
         <v>126025</v>
       </c>
-      <c r="I5" s="44">
+      <c r="I5" s="41">
         <f>(100/$B$8)*ABS(C5-F5)/C5</f>
         <v>0.11009174311926606</v>
       </c>
-      <c r="J5" s="43">
+      <c r="J5" s="40">
         <f>(1/$B$8)*ABS(C5-F5)</f>
         <v>24</v>
       </c>
-      <c r="K5" s="43">
+      <c r="K5" s="40">
         <f>(1/$B$8)*ABS(C5-F5)^2</f>
         <v>2880</v>
       </c>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="35">
+      <c r="A6" s="32">
         <v>2025</v>
       </c>
-      <c r="B6" s="35">
+      <c r="B6" s="32">
         <v>5</v>
       </c>
-      <c r="C6" s="35">
+      <c r="C6" s="32">
         <v>21725</v>
       </c>
-      <c r="D6" s="35">
+      <c r="D6" s="32">
         <f t="shared" si="0"/>
         <v>108625</v>
       </c>
-      <c r="E6" s="35">
+      <c r="E6" s="32">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="F6" s="43">
+      <c r="F6" s="40">
         <f>-235*B6+22860</f>
         <v>21685</v>
       </c>
-      <c r="G6" s="43">
+      <c r="G6" s="40">
         <f t="shared" si="2"/>
         <v>1600</v>
       </c>
-      <c r="H6" s="43">
+      <c r="H6" s="40">
         <f t="shared" si="3"/>
         <v>184900</v>
       </c>
-      <c r="I6" s="44">
+      <c r="I6" s="41">
         <f>(100/$B$8)*ABS(C6-F6)/C6</f>
         <v>3.6823935558112773E-2</v>
       </c>
-      <c r="J6" s="43">
+      <c r="J6" s="40">
         <f>(1/$B$8)*ABS(C6-F6)</f>
         <v>8</v>
       </c>
-      <c r="K6" s="43">
+      <c r="K6" s="40">
         <f>(1/$B$8)*ABS(C6-F6)^2</f>
         <v>320</v>
       </c>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="36">
+      <c r="B7" s="33">
         <f>SUM(B2:B6)</f>
         <v>15</v>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="33">
         <f>SUM(C2:C6)</f>
         <v>110775</v>
       </c>
-      <c r="D7" s="36">
+      <c r="D7" s="33">
         <f>SUM(D2:D6)</f>
         <v>329975</v>
       </c>
-      <c r="E7" s="36">
+      <c r="E7" s="33">
         <f>SUM(E2:E6)</f>
         <v>55</v>
       </c>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45">
+      <c r="F7" s="42"/>
+      <c r="G7" s="42">
         <f>SUM(G2:G6)</f>
         <v>25750</v>
       </c>
-      <c r="H7" s="45">
+      <c r="H7" s="42">
         <f>SUM(H2:H6)</f>
         <v>578000</v>
       </c>
-      <c r="I7" s="37">
+      <c r="I7" s="34">
         <f>SUM(I2:I6)</f>
         <v>0.2633614023382263</v>
       </c>
-      <c r="J7" s="45">
+      <c r="J7" s="42">
         <f>SUM(J2:J6)</f>
         <v>58</v>
       </c>
-      <c r="K7" s="45">
+      <c r="K7" s="42">
         <f>SUM(K2:K6)</f>
         <v>5150</v>
       </c>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="B8" s="38">
+      <c r="B8" s="35">
         <f>COUNT(B2:B6)</f>
         <v>5</v>
       </c>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="46"/>
-      <c r="G8" s="46"/>
-      <c r="H8" s="46"/>
-      <c r="I8" s="46"/>
-      <c r="J8" s="46"/>
-      <c r="K8" s="46"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="43"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="38">
+      <c r="B9" s="35">
         <f>AVERAGE(C2:C6)</f>
         <v>22155</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="46"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="46"/>
-      <c r="I9" s="46"/>
-      <c r="J9" s="46"/>
-      <c r="K9" s="46"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="43"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="43"/>
+      <c r="K9" s="43"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="39" t="s">
+      <c r="A10" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="B10" s="39">
+      <c r="B10" s="36">
         <f>(B8*D7-B7*C7)/(B8*E7-B7^2)</f>
         <v>-235</v>
       </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="46" t="s">
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="43" t="s">
         <v>102</v>
       </c>
-      <c r="G10" s="46">
+      <c r="G10" s="43">
         <f>1-(G7/H7)</f>
         <v>0.95544982698961933</v>
       </c>
-      <c r="H10" s="46"/>
-      <c r="I10" s="46"/>
-      <c r="J10" s="46"/>
-      <c r="K10" s="46"/>
+      <c r="H10" s="43"/>
+      <c r="I10" s="43"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="43"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="39">
+      <c r="B11" s="36">
         <f>(C7-B10*B7)/(B8)</f>
         <v>22860</v>
       </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="46"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="46"/>
-      <c r="I11" s="46"/>
-      <c r="J11" s="46"/>
-      <c r="K11" s="46"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
+      <c r="I11" s="43"/>
+      <c r="J11" s="43"/>
+      <c r="K11" s="43"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="40"/>
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="47"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="47"/>
-      <c r="J12" s="47"/>
-      <c r="K12" s="47"/>
+      <c r="A12" s="37"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="44"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="41" t="s">
+      <c r="A13" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="47"/>
-      <c r="G13" s="47"/>
-      <c r="H13" s="47"/>
-      <c r="I13" s="47"/>
-      <c r="J13" s="47"/>
-      <c r="K13" s="47"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="41" t="str">
+      <c r="A14" s="38" t="str">
         <f>"y = "&amp;B11&amp;"+"&amp;B10&amp;"x"</f>
         <v>y = 22860+-235x</v>
       </c>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="47"/>
-      <c r="I14" s="47"/>
-      <c r="J14" s="47"/>
-      <c r="K14" s="47"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="41" t="str">
+      <c r="A15" s="38" t="str">
         <f>"y = "&amp;B11+B10*(6)</f>
         <v>y = 21450</v>
       </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="47"/>
-      <c r="G15" s="47"/>
-      <c r="H15" s="47"/>
-      <c r="I15" s="47"/>
-      <c r="J15" s="47"/>
-      <c r="K15" s="47"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="44"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{600CBCD3-146A-42A4-83C6-0EE593AA074C}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="39"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="39" t="s">
+        <v>105</v>
+      </c>
+      <c r="B1" s="39" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="39">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="39">
+        <v>25</v>
+      </c>
+      <c r="B3" s="39">
+        <f>A3-A2</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="39">
+        <v>27</v>
+      </c>
+      <c r="B4" s="39">
+        <f t="shared" ref="B4:D10" si="0">A4-A3</f>
+        <v>2</v>
+      </c>
+      <c r="C4" s="39">
+        <f>B4-B3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="39">
+        <v>32</v>
+      </c>
+      <c r="B5" s="39">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="C5" s="39">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="D5" s="39">
+        <f>C5-C4</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="39">
+        <v>33</v>
+      </c>
+      <c r="B6" s="39">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C6" s="39">
+        <f t="shared" si="0"/>
+        <v>-4</v>
+      </c>
+      <c r="D6" s="39">
+        <f t="shared" si="0"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="39">
+        <v>37</v>
+      </c>
+      <c r="B7" s="39">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C7" s="39">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="D7" s="39">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="39">
+        <v>42</v>
+      </c>
+      <c r="B8" s="39">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="C8" s="39">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D8" s="39">
+        <f t="shared" si="0"/>
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="39">
+        <v>45</v>
+      </c>
+      <c r="B9" s="39">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="C9" s="39">
+        <f t="shared" si="0"/>
+        <v>-2</v>
+      </c>
+      <c r="D9" s="39">
+        <f t="shared" si="0"/>
+        <v>-3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5533,17 +5673,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="46" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
     </row>
     <row r="2" spans="1:9">
       <c r="B2" t="s">
@@ -5575,7 +5715,7 @@
       <c r="E3" s="28">
         <v>3.5</v>
       </c>
-      <c r="G3" s="33" t="s">
+      <c r="G3" s="45" t="s">
         <v>43</v>
       </c>
       <c r="H3" t="s">
@@ -5602,7 +5742,7 @@
       <c r="E4" s="28">
         <v>3.6</v>
       </c>
-      <c r="G4" s="33"/>
+      <c r="G4" s="45"/>
       <c r="H4" t="s">
         <v>24</v>
       </c>
@@ -5627,7 +5767,7 @@
       <c r="E5" s="28">
         <v>3.1</v>
       </c>
-      <c r="G5" s="33"/>
+      <c r="G5" s="45"/>
       <c r="H5" t="s">
         <v>26</v>
       </c>
@@ -5652,7 +5792,7 @@
       <c r="E6" s="28">
         <v>4</v>
       </c>
-      <c r="G6" s="33"/>
+      <c r="G6" s="45"/>
       <c r="H6" t="s">
         <v>28</v>
       </c>
@@ -5699,17 +5839,17 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="15">
-      <c r="A12" s="34" t="s">
+      <c r="A12" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="34"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
+      <c r="B12" s="46"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="46"/>
+      <c r="I12" s="46"/>
     </row>
     <row r="14" spans="1:9">
       <c r="B14" t="s">
@@ -5810,17 +5950,17 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="15">
-      <c r="A21" s="34" t="s">
+      <c r="A21" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="B21" s="34"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="29" t="s">
@@ -5905,17 +6045,17 @@
       </c>
     </row>
     <row r="28" spans="1:9" ht="15">
-      <c r="A28" s="34" t="s">
+      <c r="A28" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
+      <c r="B28" s="46"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="46"/>
+      <c r="I28" s="46"/>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="29" t="s">
@@ -6041,19 +6181,19 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:11" ht="15">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="29" t="s">
@@ -6092,7 +6232,7 @@
       <c r="E3" s="29"/>
       <c r="F3" s="29"/>
       <c r="G3" s="29"/>
-      <c r="H3" s="33" t="s">
+      <c r="H3" s="45" t="s">
         <v>72</v>
       </c>
       <c r="I3" s="29" t="s">
@@ -6122,7 +6262,7 @@
       <c r="E4" s="29"/>
       <c r="F4" s="29"/>
       <c r="G4" s="29"/>
-      <c r="H4" s="33"/>
+      <c r="H4" s="45"/>
       <c r="I4" s="29" t="s">
         <v>24</v>
       </c>
@@ -6150,7 +6290,7 @@
       <c r="E5" s="29"/>
       <c r="F5" s="29"/>
       <c r="G5" s="29"/>
-      <c r="H5" s="33"/>
+      <c r="H5" s="45"/>
       <c r="I5" s="29" t="s">
         <v>26</v>
       </c>
@@ -6178,7 +6318,7 @@
       <c r="E6" s="29"/>
       <c r="F6" s="29"/>
       <c r="G6" s="29"/>
-      <c r="H6" s="33"/>
+      <c r="H6" s="45"/>
       <c r="I6" s="29" t="s">
         <v>28</v>
       </c>
@@ -6253,7 +6393,7 @@
       <c r="F9" s="29"/>
       <c r="G9" s="29"/>
       <c r="H9" s="29"/>
-      <c r="I9" s="33" t="s">
+      <c r="I9" s="45" t="s">
         <v>43</v>
       </c>
       <c r="J9" s="29" t="s">
@@ -6283,7 +6423,7 @@
       <c r="F10" s="29"/>
       <c r="G10" s="29"/>
       <c r="H10" s="29"/>
-      <c r="I10" s="33"/>
+      <c r="I10" s="45"/>
       <c r="J10" s="29" t="s">
         <v>24</v>
       </c>
@@ -6311,7 +6451,7 @@
       <c r="F11" s="29"/>
       <c r="G11" s="29"/>
       <c r="H11" s="29"/>
-      <c r="I11" s="33"/>
+      <c r="I11" s="45"/>
       <c r="J11" s="29" t="s">
         <v>26</v>
       </c>
@@ -6339,7 +6479,7 @@
       <c r="F12" s="29"/>
       <c r="G12" s="29"/>
       <c r="H12" s="29"/>
-      <c r="I12" s="33"/>
+      <c r="I12" s="45"/>
       <c r="J12" s="29" t="s">
         <v>28</v>
       </c>
@@ -6442,17 +6582,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="45" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="45" t="s">
         <v>74</v>
       </c>
       <c r="B2" s="26" t="s">
@@ -6463,7 +6603,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="33"/>
+      <c r="A3" s="45"/>
       <c r="B3" s="26" t="s">
         <v>24</v>
       </c>
@@ -6472,7 +6612,7 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="33"/>
+      <c r="A4" s="45"/>
       <c r="B4" s="26" t="s">
         <v>26</v>
       </c>
@@ -6481,7 +6621,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="33"/>
+      <c r="A5" s="45"/>
       <c r="B5" s="26" t="s">
         <v>28</v>
       </c>
@@ -6490,7 +6630,7 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="45" t="s">
         <v>75</v>
       </c>
       <c r="B6" s="26" t="s">
@@ -6501,7 +6641,7 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="33"/>
+      <c r="A7" s="45"/>
       <c r="B7" s="26" t="s">
         <v>24</v>
       </c>
@@ -6513,7 +6653,7 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="33"/>
+      <c r="A8" s="45"/>
       <c r="B8" s="26" t="s">
         <v>26</v>
       </c>
@@ -6522,7 +6662,7 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="33"/>
+      <c r="A9" s="45"/>
       <c r="B9" s="26" t="s">
         <v>28</v>
       </c>

</xml_diff>